<commit_message>
Code review fixes: security hardening, id/compact/audit/undo bugs, i18n, E2E regression tests, docs
</commit_message>
<xml_diff>
--- a/output/asset-inventory-zh.xlsx
+++ b/output/asset-inventory-zh.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="全部资产" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="按类别" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="摘要" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="访问信息" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="财务摘要" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="保险" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="受益人" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="遗产" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="全部资产" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="按类别" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="摘要" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="访问信息" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="财务摘要" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="保险" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="受益人" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="遗产" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -602,7 +602,7 @@
       </c>
       <c r="P2" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q2" t="inlineStr"/>
@@ -659,7 +659,7 @@
       </c>
       <c r="P3" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q3" t="inlineStr"/>
@@ -716,7 +716,7 @@
       </c>
       <c r="P4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q4" t="inlineStr"/>
@@ -773,7 +773,7 @@
       </c>
       <c r="P5" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q5" t="inlineStr"/>
@@ -826,7 +826,7 @@
       </c>
       <c r="P6" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q6" t="inlineStr"/>
@@ -883,7 +883,7 @@
       </c>
       <c r="P7" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q7" t="inlineStr"/>
@@ -936,7 +936,7 @@
       </c>
       <c r="P8" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q8" t="inlineStr"/>
@@ -989,7 +989,7 @@
       </c>
       <c r="P9" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q9" t="inlineStr"/>
@@ -1046,7 +1046,7 @@
       </c>
       <c r="P10" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q10" t="inlineStr"/>
@@ -1103,7 +1103,7 @@
       </c>
       <c r="P11" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q11" t="inlineStr"/>
@@ -1160,7 +1160,7 @@
       </c>
       <c r="P12" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q12" t="inlineStr"/>
@@ -1217,7 +1217,7 @@
       </c>
       <c r="P13" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q13" t="inlineStr"/>
@@ -1274,7 +1274,7 @@
       </c>
       <c r="P14" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q14" t="inlineStr"/>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="P15" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q15" t="inlineStr"/>
@@ -1388,7 +1388,7 @@
       </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q16" t="inlineStr"/>
@@ -1445,7 +1445,7 @@
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q17" t="inlineStr"/>
@@ -1502,7 +1502,7 @@
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q18" t="inlineStr"/>
@@ -1559,7 +1559,7 @@
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q19" t="inlineStr"/>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q20" t="inlineStr"/>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="P21" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q21" t="inlineStr"/>
@@ -1730,7 +1730,7 @@
       </c>
       <c r="P22" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q22" t="inlineStr"/>
@@ -1787,7 +1787,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q23" t="inlineStr"/>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q24" t="inlineStr"/>
@@ -1901,7 +1901,7 @@
       </c>
       <c r="P25" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q25" t="inlineStr"/>
@@ -1958,7 +1958,7 @@
       </c>
       <c r="P26" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q26" t="inlineStr"/>
@@ -2015,7 +2015,7 @@
       </c>
       <c r="P27" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q27" t="inlineStr"/>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="P28" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q28" t="inlineStr"/>
@@ -2129,7 +2129,7 @@
       </c>
       <c r="P29" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q29" t="inlineStr"/>
@@ -2186,7 +2186,7 @@
       </c>
       <c r="P30" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q30" t="inlineStr"/>
@@ -2243,7 +2243,7 @@
       </c>
       <c r="P31" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q31" t="inlineStr"/>
@@ -2300,7 +2300,7 @@
       </c>
       <c r="P32" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q32" t="inlineStr"/>
@@ -2357,7 +2357,7 @@
       </c>
       <c r="P33" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q33" t="inlineStr"/>
@@ -2414,7 +2414,7 @@
       </c>
       <c r="P34" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q34" t="inlineStr"/>
@@ -2471,7 +2471,7 @@
       </c>
       <c r="P35" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q35" t="inlineStr"/>
@@ -2528,7 +2528,7 @@
       </c>
       <c r="P36" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q36" t="inlineStr"/>
@@ -2585,7 +2585,7 @@
       </c>
       <c r="P37" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q37" t="inlineStr"/>
@@ -2642,7 +2642,7 @@
       </c>
       <c r="P38" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q38" t="inlineStr"/>
@@ -2699,7 +2699,7 @@
       </c>
       <c r="P39" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q39" t="inlineStr"/>
@@ -2756,7 +2756,7 @@
       </c>
       <c r="P40" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q40" t="inlineStr"/>
@@ -2813,7 +2813,7 @@
       </c>
       <c r="P41" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q41" t="inlineStr"/>
@@ -2870,7 +2870,7 @@
       </c>
       <c r="P42" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q42" t="inlineStr"/>
@@ -2927,7 +2927,7 @@
       </c>
       <c r="P43" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q43" t="inlineStr"/>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="P44" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q44" t="inlineStr"/>
@@ -3041,7 +3041,7 @@
       </c>
       <c r="P45" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q45" t="inlineStr"/>
@@ -3098,7 +3098,7 @@
       </c>
       <c r="P46" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q46" t="inlineStr"/>
@@ -3155,7 +3155,7 @@
       </c>
       <c r="P47" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q47" t="inlineStr"/>
@@ -3212,7 +3212,7 @@
       </c>
       <c r="P48" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q48" t="inlineStr"/>
@@ -3269,7 +3269,7 @@
       </c>
       <c r="P49" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q49" t="inlineStr"/>
@@ -3326,7 +3326,7 @@
       </c>
       <c r="P50" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q50" t="inlineStr"/>
@@ -3383,7 +3383,7 @@
       </c>
       <c r="P51" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q51" t="inlineStr"/>
@@ -3440,7 +3440,7 @@
       </c>
       <c r="P52" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q52" t="inlineStr"/>
@@ -3497,7 +3497,7 @@
       </c>
       <c r="P53" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q53" t="inlineStr"/>
@@ -3554,7 +3554,7 @@
       </c>
       <c r="P54" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q54" t="inlineStr"/>
@@ -3611,7 +3611,7 @@
       </c>
       <c r="P55" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q55" t="inlineStr"/>
@@ -3668,7 +3668,7 @@
       </c>
       <c r="P56" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q56" t="inlineStr"/>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="P57" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q57" t="inlineStr"/>
@@ -3782,7 +3782,7 @@
       </c>
       <c r="P58" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q58" t="inlineStr"/>
@@ -3839,7 +3839,7 @@
       </c>
       <c r="P59" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q59" t="inlineStr"/>
@@ -3896,7 +3896,7 @@
       </c>
       <c r="P60" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q60" t="inlineStr"/>
@@ -3953,7 +3953,7 @@
       </c>
       <c r="P61" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q61" t="inlineStr"/>
@@ -4010,7 +4010,7 @@
       </c>
       <c r="P62" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q62" t="inlineStr"/>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="P63" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q63" t="inlineStr"/>
@@ -4124,7 +4124,7 @@
       </c>
       <c r="P64" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q64" t="inlineStr"/>
@@ -4181,7 +4181,7 @@
       </c>
       <c r="P65" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q65" t="inlineStr"/>
@@ -4238,7 +4238,7 @@
       </c>
       <c r="P66" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q66" t="inlineStr"/>
@@ -4295,7 +4295,7 @@
       </c>
       <c r="P67" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q67" t="inlineStr"/>
@@ -4352,7 +4352,7 @@
       </c>
       <c r="P68" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q68" t="inlineStr"/>
@@ -4409,7 +4409,7 @@
       </c>
       <c r="P69" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q69" t="inlineStr"/>
@@ -4466,7 +4466,7 @@
       </c>
       <c r="P70" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q70" t="inlineStr"/>
@@ -4523,7 +4523,7 @@
       </c>
       <c r="P71" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q71" t="inlineStr"/>
@@ -4580,7 +4580,7 @@
       </c>
       <c r="P72" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q72" t="inlineStr"/>
@@ -4637,7 +4637,7 @@
       </c>
       <c r="P73" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q73" t="inlineStr"/>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="P74" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q74" t="inlineStr"/>
@@ -4751,7 +4751,7 @@
       </c>
       <c r="P75" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q75" t="inlineStr"/>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="P76" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q76" t="inlineStr"/>
@@ -4865,7 +4865,7 @@
       </c>
       <c r="P77" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q77" t="inlineStr"/>
@@ -4922,7 +4922,7 @@
       </c>
       <c r="P78" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q78" t="inlineStr"/>
@@ -4979,7 +4979,7 @@
       </c>
       <c r="P79" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q79" t="inlineStr"/>
@@ -5036,7 +5036,7 @@
       </c>
       <c r="P80" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q80" t="inlineStr"/>
@@ -5093,7 +5093,7 @@
       </c>
       <c r="P81" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q81" t="inlineStr"/>
@@ -5150,7 +5150,7 @@
       </c>
       <c r="P82" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q82" t="inlineStr"/>
@@ -5207,7 +5207,7 @@
       </c>
       <c r="P83" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q83" t="inlineStr"/>
@@ -5264,7 +5264,7 @@
       </c>
       <c r="P84" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q84" t="inlineStr"/>
@@ -5321,7 +5321,7 @@
       </c>
       <c r="P85" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q85" t="inlineStr"/>
@@ -5378,7 +5378,7 @@
       </c>
       <c r="P86" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q86" t="inlineStr"/>
@@ -5435,7 +5435,7 @@
       </c>
       <c r="P87" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q87" t="inlineStr"/>
@@ -5492,7 +5492,7 @@
       </c>
       <c r="P88" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q88" t="inlineStr"/>
@@ -5549,7 +5549,7 @@
       </c>
       <c r="P89" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q89" t="inlineStr"/>
@@ -5606,7 +5606,7 @@
       </c>
       <c r="P90" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q90" t="inlineStr"/>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="P91" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q91" t="inlineStr"/>
@@ -5720,7 +5720,7 @@
       </c>
       <c r="P92" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q92" t="inlineStr"/>
@@ -5777,7 +5777,7 @@
       </c>
       <c r="P93" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q93" t="inlineStr"/>
@@ -5834,7 +5834,7 @@
       </c>
       <c r="P94" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q94" t="inlineStr"/>
@@ -5891,7 +5891,7 @@
       </c>
       <c r="P95" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q95" t="inlineStr"/>
@@ -5948,7 +5948,7 @@
       </c>
       <c r="P96" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q96" t="inlineStr"/>
@@ -6005,7 +6005,7 @@
       </c>
       <c r="P97" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q97" t="inlineStr"/>
@@ -6062,7 +6062,7 @@
       </c>
       <c r="P98" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q98" t="inlineStr"/>
@@ -6119,7 +6119,7 @@
       </c>
       <c r="P99" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q99" t="inlineStr"/>
@@ -6176,7 +6176,7 @@
       </c>
       <c r="P100" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q100" t="inlineStr"/>
@@ -6233,7 +6233,7 @@
       </c>
       <c r="P101" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q101" t="inlineStr"/>
@@ -6290,7 +6290,7 @@
       </c>
       <c r="P102" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q102" t="inlineStr"/>
@@ -6347,7 +6347,7 @@
       </c>
       <c r="P103" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q103" t="inlineStr"/>
@@ -6404,7 +6404,7 @@
       </c>
       <c r="P104" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q104" t="inlineStr"/>
@@ -6461,7 +6461,7 @@
       </c>
       <c r="P105" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q105" t="inlineStr"/>
@@ -6518,7 +6518,7 @@
       </c>
       <c r="P106" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q106" t="inlineStr"/>
@@ -6575,7 +6575,7 @@
       </c>
       <c r="P107" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q107" t="inlineStr"/>
@@ -6632,7 +6632,7 @@
       </c>
       <c r="P108" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q108" t="inlineStr"/>
@@ -6689,7 +6689,7 @@
       </c>
       <c r="P109" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q109" t="inlineStr"/>
@@ -6746,7 +6746,7 @@
       </c>
       <c r="P110" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q110" t="inlineStr"/>
@@ -6803,7 +6803,7 @@
       </c>
       <c r="P111" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q111" t="inlineStr"/>
@@ -6860,7 +6860,7 @@
       </c>
       <c r="P112" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q112" t="inlineStr"/>
@@ -6913,7 +6913,7 @@
       </c>
       <c r="P113" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q113" t="inlineStr"/>
@@ -6966,7 +6966,7 @@
       </c>
       <c r="P114" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q114" t="inlineStr"/>
@@ -7019,7 +7019,7 @@
       </c>
       <c r="P115" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q115" t="inlineStr"/>
@@ -7072,7 +7072,7 @@
       </c>
       <c r="P116" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q116" t="inlineStr"/>
@@ -7125,7 +7125,7 @@
       </c>
       <c r="P117" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q117" t="inlineStr"/>
@@ -7178,7 +7178,7 @@
       </c>
       <c r="P118" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q118" t="inlineStr"/>
@@ -7231,7 +7231,7 @@
       </c>
       <c r="P119" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q119" t="inlineStr"/>
@@ -7288,7 +7288,7 @@
       </c>
       <c r="P120" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q120" t="inlineStr"/>
@@ -7341,7 +7341,7 @@
       </c>
       <c r="P121" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q121" t="inlineStr"/>
@@ -7398,7 +7398,7 @@
       </c>
       <c r="P122" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q122" t="inlineStr"/>
@@ -7455,7 +7455,7 @@
       </c>
       <c r="P123" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q123" t="inlineStr"/>
@@ -7512,7 +7512,7 @@
       </c>
       <c r="P124" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q124" t="inlineStr"/>
@@ -7565,7 +7565,7 @@
       </c>
       <c r="P125" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q125" t="inlineStr"/>
@@ -7618,7 +7618,7 @@
       </c>
       <c r="P126" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q126" t="inlineStr"/>
@@ -7671,7 +7671,7 @@
       </c>
       <c r="P127" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q127" t="inlineStr"/>
@@ -7724,7 +7724,7 @@
       </c>
       <c r="P128" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q128" t="inlineStr"/>
@@ -7777,7 +7777,7 @@
       </c>
       <c r="P129" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q129" t="inlineStr"/>
@@ -7830,7 +7830,7 @@
       </c>
       <c r="P130" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q130" t="inlineStr"/>
@@ -7883,7 +7883,7 @@
       </c>
       <c r="P131" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q131" t="inlineStr"/>
@@ -7936,7 +7936,7 @@
       </c>
       <c r="P132" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q132" t="inlineStr"/>
@@ -7989,7 +7989,7 @@
       </c>
       <c r="P133" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q133" t="inlineStr"/>
@@ -8042,7 +8042,7 @@
       </c>
       <c r="P134" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q134" t="inlineStr"/>
@@ -8095,7 +8095,7 @@
       </c>
       <c r="P135" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q135" t="inlineStr"/>
@@ -8148,7 +8148,7 @@
       </c>
       <c r="P136" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q136" t="inlineStr"/>
@@ -8201,7 +8201,7 @@
       </c>
       <c r="P137" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q137" t="inlineStr"/>
@@ -8254,7 +8254,7 @@
       </c>
       <c r="P138" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q138" t="inlineStr"/>
@@ -8307,7 +8307,7 @@
       </c>
       <c r="P139" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q139" t="inlineStr"/>
@@ -8360,7 +8360,7 @@
       </c>
       <c r="P140" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q140" t="inlineStr"/>
@@ -8413,7 +8413,7 @@
       </c>
       <c r="P141" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q141" t="inlineStr"/>
@@ -8466,7 +8466,7 @@
       </c>
       <c r="P142" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q142" t="inlineStr"/>
@@ -8519,7 +8519,7 @@
       </c>
       <c r="P143" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q143" t="inlineStr"/>
@@ -8572,7 +8572,7 @@
       </c>
       <c r="P144" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q144" t="inlineStr"/>
@@ -8625,7 +8625,7 @@
       </c>
       <c r="P145" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q145" t="inlineStr"/>
@@ -8678,7 +8678,7 @@
       </c>
       <c r="P146" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q146" t="inlineStr"/>
@@ -8731,7 +8731,7 @@
       </c>
       <c r="P147" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q147" t="inlineStr"/>
@@ -8784,7 +8784,7 @@
       </c>
       <c r="P148" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q148" t="inlineStr"/>
@@ -8837,7 +8837,7 @@
       </c>
       <c r="P149" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q149" t="inlineStr"/>
@@ -8890,7 +8890,7 @@
       </c>
       <c r="P150" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q150" t="inlineStr"/>
@@ -8947,7 +8947,7 @@
       </c>
       <c r="P151" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q151" t="inlineStr"/>
@@ -9000,7 +9000,7 @@
       </c>
       <c r="P152" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q152" t="inlineStr"/>
@@ -9053,7 +9053,7 @@
       </c>
       <c r="P153" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q153" t="inlineStr"/>
@@ -9106,7 +9106,7 @@
       </c>
       <c r="P154" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q154" t="inlineStr"/>
@@ -9159,7 +9159,7 @@
       </c>
       <c r="P155" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q155" t="inlineStr"/>
@@ -9212,7 +9212,7 @@
       </c>
       <c r="P156" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q156" t="inlineStr"/>
@@ -9265,7 +9265,7 @@
       </c>
       <c r="P157" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q157" t="inlineStr"/>
@@ -9318,7 +9318,7 @@
       </c>
       <c r="P158" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q158" t="inlineStr"/>
@@ -9371,7 +9371,7 @@
       </c>
       <c r="P159" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q159" t="inlineStr"/>
@@ -9424,7 +9424,7 @@
       </c>
       <c r="P160" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q160" t="inlineStr"/>
@@ -9477,7 +9477,7 @@
       </c>
       <c r="P161" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q161" t="inlineStr"/>
@@ -9530,7 +9530,7 @@
       </c>
       <c r="P162" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q162" t="inlineStr"/>
@@ -9583,7 +9583,7 @@
       </c>
       <c r="P163" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q163" t="inlineStr"/>
@@ -9636,7 +9636,7 @@
       </c>
       <c r="P164" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q164" t="inlineStr"/>
@@ -9689,7 +9689,7 @@
       </c>
       <c r="P165" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q165" t="inlineStr"/>
@@ -9742,7 +9742,7 @@
       </c>
       <c r="P166" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q166" t="inlineStr"/>
@@ -9795,7 +9795,7 @@
       </c>
       <c r="P167" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q167" t="inlineStr"/>
@@ -9848,7 +9848,7 @@
       </c>
       <c r="P168" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q168" t="inlineStr"/>
@@ -9901,7 +9901,7 @@
       </c>
       <c r="P169" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q169" t="inlineStr"/>
@@ -9954,7 +9954,7 @@
       </c>
       <c r="P170" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q170" t="inlineStr"/>
@@ -10011,7 +10011,7 @@
       </c>
       <c r="P171" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q171" t="inlineStr"/>
@@ -10068,7 +10068,7 @@
       </c>
       <c r="P172" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q172" t="inlineStr"/>
@@ -10125,7 +10125,7 @@
       </c>
       <c r="P173" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q173" t="inlineStr"/>
@@ -10182,7 +10182,7 @@
       </c>
       <c r="P174" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q174" t="inlineStr"/>
@@ -10239,7 +10239,7 @@
       </c>
       <c r="P175" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q175" t="inlineStr"/>
@@ -10296,7 +10296,7 @@
       </c>
       <c r="P176" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q176" t="inlineStr"/>
@@ -10353,7 +10353,7 @@
       </c>
       <c r="P177" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q177" t="inlineStr"/>
@@ -10410,7 +10410,7 @@
       </c>
       <c r="P178" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q178" t="inlineStr"/>
@@ -10467,7 +10467,7 @@
       </c>
       <c r="P179" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q179" t="inlineStr"/>
@@ -10524,7 +10524,7 @@
       </c>
       <c r="P180" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q180" t="inlineStr"/>
@@ -10581,7 +10581,7 @@
       </c>
       <c r="P181" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q181" t="inlineStr"/>
@@ -10638,7 +10638,7 @@
       </c>
       <c r="P182" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q182" t="inlineStr"/>
@@ -10695,7 +10695,7 @@
       </c>
       <c r="P183" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q183" t="inlineStr"/>
@@ -10752,7 +10752,7 @@
       </c>
       <c r="P184" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q184" t="inlineStr"/>
@@ -10809,7 +10809,7 @@
       </c>
       <c r="P185" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q185" t="inlineStr"/>
@@ -10866,7 +10866,7 @@
       </c>
       <c r="P186" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q186" t="inlineStr"/>
@@ -10923,7 +10923,7 @@
       </c>
       <c r="P187" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q187" t="inlineStr"/>
@@ -10980,7 +10980,7 @@
       </c>
       <c r="P188" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q188" t="inlineStr"/>
@@ -11037,7 +11037,7 @@
       </c>
       <c r="P189" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q189" t="inlineStr"/>
@@ -11094,7 +11094,7 @@
       </c>
       <c r="P190" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q190" t="inlineStr"/>
@@ -11151,7 +11151,7 @@
       </c>
       <c r="P191" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q191" t="inlineStr"/>
@@ -11208,7 +11208,7 @@
       </c>
       <c r="P192" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q192" t="inlineStr"/>
@@ -11265,7 +11265,7 @@
       </c>
       <c r="P193" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q193" t="inlineStr"/>
@@ -11322,7 +11322,7 @@
       </c>
       <c r="P194" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q194" t="inlineStr"/>
@@ -11379,7 +11379,7 @@
       </c>
       <c r="P195" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q195" t="inlineStr"/>
@@ -11436,7 +11436,7 @@
       </c>
       <c r="P196" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q196" t="inlineStr"/>
@@ -11493,7 +11493,7 @@
       </c>
       <c r="P197" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q197" t="inlineStr"/>
@@ -11550,7 +11550,7 @@
       </c>
       <c r="P198" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q198" t="inlineStr"/>
@@ -11607,7 +11607,7 @@
       </c>
       <c r="P199" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q199" t="inlineStr"/>
@@ -11664,7 +11664,7 @@
       </c>
       <c r="P200" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q200" t="inlineStr"/>
@@ -11721,7 +11721,7 @@
       </c>
       <c r="P201" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q201" t="inlineStr"/>
@@ -11778,7 +11778,7 @@
       </c>
       <c r="P202" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q202" t="inlineStr"/>
@@ -11835,7 +11835,7 @@
       </c>
       <c r="P203" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q203" t="inlineStr"/>
@@ -11892,7 +11892,7 @@
       </c>
       <c r="P204" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q204" t="inlineStr"/>
@@ -11949,7 +11949,7 @@
       </c>
       <c r="P205" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q205" t="inlineStr"/>
@@ -12006,7 +12006,7 @@
       </c>
       <c r="P206" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q206" t="inlineStr"/>
@@ -12063,7 +12063,7 @@
       </c>
       <c r="P207" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q207" t="inlineStr"/>
@@ -12120,7 +12120,7 @@
       </c>
       <c r="P208" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q208" t="inlineStr"/>
@@ -12177,7 +12177,7 @@
       </c>
       <c r="P209" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q209" t="inlineStr"/>
@@ -12234,7 +12234,7 @@
       </c>
       <c r="P210" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q210" t="inlineStr"/>
@@ -12291,7 +12291,7 @@
       </c>
       <c r="P211" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q211" t="inlineStr"/>
@@ -12348,7 +12348,7 @@
       </c>
       <c r="P212" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q212" t="inlineStr"/>
@@ -12405,7 +12405,7 @@
       </c>
       <c r="P213" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q213" t="inlineStr"/>
@@ -12462,7 +12462,7 @@
       </c>
       <c r="P214" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q214" t="inlineStr"/>
@@ -12519,7 +12519,7 @@
       </c>
       <c r="P215" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q215" t="inlineStr"/>
@@ -12576,7 +12576,7 @@
       </c>
       <c r="P216" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q216" t="inlineStr"/>
@@ -12633,7 +12633,7 @@
       </c>
       <c r="P217" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q217" t="inlineStr"/>
@@ -12690,7 +12690,7 @@
       </c>
       <c r="P218" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q218" t="inlineStr"/>
@@ -12747,7 +12747,7 @@
       </c>
       <c r="P219" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q219" t="inlineStr"/>
@@ -12804,7 +12804,7 @@
       </c>
       <c r="P220" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q220" t="inlineStr"/>
@@ -12861,7 +12861,7 @@
       </c>
       <c r="P221" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q221" t="inlineStr"/>
@@ -12918,7 +12918,7 @@
       </c>
       <c r="P222" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q222" t="inlineStr"/>
@@ -12975,7 +12975,7 @@
       </c>
       <c r="P223" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q223" t="inlineStr"/>
@@ -13032,7 +13032,7 @@
       </c>
       <c r="P224" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q224" t="inlineStr"/>
@@ -13089,7 +13089,7 @@
       </c>
       <c r="P225" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q225" t="inlineStr"/>
@@ -13146,7 +13146,7 @@
       </c>
       <c r="P226" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q226" t="inlineStr"/>
@@ -13203,7 +13203,7 @@
       </c>
       <c r="P227" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q227" t="inlineStr"/>
@@ -13260,7 +13260,7 @@
       </c>
       <c r="P228" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q228" t="inlineStr"/>
@@ -13317,7 +13317,7 @@
       </c>
       <c r="P229" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q229" t="inlineStr"/>
@@ -13374,7 +13374,7 @@
       </c>
       <c r="P230" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q230" t="inlineStr"/>
@@ -13431,7 +13431,7 @@
       </c>
       <c r="P231" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q231" t="inlineStr"/>
@@ -13488,7 +13488,7 @@
       </c>
       <c r="P232" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q232" t="inlineStr"/>
@@ -13545,7 +13545,7 @@
       </c>
       <c r="P233" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q233" t="inlineStr"/>
@@ -13602,7 +13602,7 @@
       </c>
       <c r="P234" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q234" t="inlineStr"/>
@@ -13659,7 +13659,7 @@
       </c>
       <c r="P235" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q235" t="inlineStr"/>
@@ -13716,7 +13716,7 @@
       </c>
       <c r="P236" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q236" t="inlineStr"/>
@@ -13773,7 +13773,7 @@
       </c>
       <c r="P237" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q237" t="inlineStr"/>
@@ -13830,7 +13830,7 @@
       </c>
       <c r="P238" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q238" t="inlineStr"/>
@@ -13887,7 +13887,7 @@
       </c>
       <c r="P239" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q239" t="inlineStr"/>
@@ -13944,7 +13944,7 @@
       </c>
       <c r="P240" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q240" t="inlineStr"/>
@@ -14001,7 +14001,7 @@
       </c>
       <c r="P241" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q241" t="inlineStr"/>
@@ -14058,7 +14058,7 @@
       </c>
       <c r="P242" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q242" t="inlineStr"/>
@@ -14115,7 +14115,7 @@
       </c>
       <c r="P243" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q243" t="inlineStr"/>
@@ -14172,7 +14172,7 @@
       </c>
       <c r="P244" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q244" t="inlineStr"/>
@@ -14229,7 +14229,7 @@
       </c>
       <c r="P245" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q245" t="inlineStr"/>
@@ -14286,7 +14286,7 @@
       </c>
       <c r="P246" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q246" t="inlineStr"/>
@@ -14343,7 +14343,7 @@
       </c>
       <c r="P247" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q247" t="inlineStr"/>
@@ -14400,7 +14400,7 @@
       </c>
       <c r="P248" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q248" t="inlineStr"/>
@@ -14457,7 +14457,7 @@
       </c>
       <c r="P249" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q249" t="inlineStr"/>
@@ -14514,7 +14514,7 @@
       </c>
       <c r="P250" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q250" t="inlineStr"/>
@@ -14571,7 +14571,7 @@
       </c>
       <c r="P251" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q251" t="inlineStr"/>
@@ -14628,7 +14628,7 @@
       </c>
       <c r="P252" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q252" t="inlineStr"/>
@@ -14685,7 +14685,7 @@
       </c>
       <c r="P253" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q253" t="inlineStr"/>
@@ -14742,7 +14742,7 @@
       </c>
       <c r="P254" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q254" t="inlineStr"/>
@@ -14799,7 +14799,7 @@
       </c>
       <c r="P255" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q255" t="inlineStr"/>
@@ -14856,7 +14856,7 @@
       </c>
       <c r="P256" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q256" t="inlineStr"/>
@@ -14913,7 +14913,7 @@
       </c>
       <c r="P257" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q257" t="inlineStr"/>
@@ -14970,7 +14970,7 @@
       </c>
       <c r="P258" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q258" t="inlineStr"/>
@@ -15027,7 +15027,7 @@
       </c>
       <c r="P259" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q259" t="inlineStr"/>
@@ -15084,7 +15084,7 @@
       </c>
       <c r="P260" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q260" t="inlineStr"/>
@@ -15141,7 +15141,7 @@
       </c>
       <c r="P261" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q261" t="inlineStr"/>
@@ -15198,7 +15198,7 @@
       </c>
       <c r="P262" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q262" t="inlineStr"/>
@@ -15255,7 +15255,7 @@
       </c>
       <c r="P263" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q263" t="inlineStr"/>
@@ -15312,7 +15312,7 @@
       </c>
       <c r="P264" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q264" t="inlineStr"/>
@@ -15369,7 +15369,7 @@
       </c>
       <c r="P265" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q265" t="inlineStr"/>
@@ -15426,7 +15426,7 @@
       </c>
       <c r="P266" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q266" t="inlineStr"/>
@@ -15483,7 +15483,7 @@
       </c>
       <c r="P267" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q267" t="inlineStr"/>
@@ -15540,7 +15540,7 @@
       </c>
       <c r="P268" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q268" t="inlineStr"/>
@@ -15597,7 +15597,7 @@
       </c>
       <c r="P269" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q269" t="inlineStr"/>
@@ -15654,7 +15654,7 @@
       </c>
       <c r="P270" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q270" t="inlineStr"/>
@@ -15711,7 +15711,7 @@
       </c>
       <c r="P271" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q271" t="inlineStr"/>
@@ -15768,7 +15768,7 @@
       </c>
       <c r="P272" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q272" t="inlineStr"/>
@@ -15825,7 +15825,7 @@
       </c>
       <c r="P273" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q273" t="inlineStr"/>
@@ -15882,7 +15882,7 @@
       </c>
       <c r="P274" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q274" t="inlineStr"/>
@@ -15939,7 +15939,7 @@
       </c>
       <c r="P275" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q275" t="inlineStr"/>
@@ -15996,7 +15996,7 @@
       </c>
       <c r="P276" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q276" t="inlineStr"/>
@@ -16053,7 +16053,7 @@
       </c>
       <c r="P277" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q277" t="inlineStr"/>
@@ -16110,7 +16110,7 @@
       </c>
       <c r="P278" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q278" t="inlineStr"/>
@@ -16167,7 +16167,7 @@
       </c>
       <c r="P279" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q279" t="inlineStr"/>
@@ -16224,7 +16224,7 @@
       </c>
       <c r="P280" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q280" t="inlineStr"/>
@@ -16281,7 +16281,7 @@
       </c>
       <c r="P281" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q281" t="inlineStr"/>
@@ -16338,7 +16338,7 @@
       </c>
       <c r="P282" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q282" t="inlineStr"/>
@@ -16395,7 +16395,7 @@
       </c>
       <c r="P283" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q283" t="inlineStr"/>
@@ -16452,7 +16452,7 @@
       </c>
       <c r="P284" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q284" t="inlineStr"/>
@@ -16509,7 +16509,7 @@
       </c>
       <c r="P285" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q285" t="inlineStr"/>
@@ -16566,7 +16566,7 @@
       </c>
       <c r="P286" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q286" t="inlineStr"/>
@@ -16623,7 +16623,7 @@
       </c>
       <c r="P287" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q287" t="inlineStr"/>
@@ -16680,7 +16680,7 @@
       </c>
       <c r="P288" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q288" t="inlineStr"/>
@@ -16737,7 +16737,7 @@
       </c>
       <c r="P289" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q289" t="inlineStr"/>
@@ -16794,7 +16794,7 @@
       </c>
       <c r="P290" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q290" t="inlineStr"/>
@@ -16851,7 +16851,7 @@
       </c>
       <c r="P291" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q291" t="inlineStr"/>
@@ -16908,7 +16908,7 @@
       </c>
       <c r="P292" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q292" t="inlineStr"/>
@@ -16965,7 +16965,7 @@
       </c>
       <c r="P293" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q293" t="inlineStr"/>
@@ -17022,7 +17022,7 @@
       </c>
       <c r="P294" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q294" t="inlineStr"/>
@@ -17079,7 +17079,7 @@
       </c>
       <c r="P295" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q295" t="inlineStr"/>
@@ -17136,7 +17136,7 @@
       </c>
       <c r="P296" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q296" t="inlineStr"/>
@@ -17193,7 +17193,7 @@
       </c>
       <c r="P297" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q297" t="inlineStr"/>
@@ -17250,7 +17250,7 @@
       </c>
       <c r="P298" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q298" t="inlineStr"/>
@@ -17307,7 +17307,7 @@
       </c>
       <c r="P299" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q299" t="inlineStr"/>
@@ -17364,7 +17364,7 @@
       </c>
       <c r="P300" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q300" t="inlineStr"/>
@@ -17421,7 +17421,7 @@
       </c>
       <c r="P301" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q301" t="inlineStr"/>
@@ -17478,7 +17478,7 @@
       </c>
       <c r="P302" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q302" t="inlineStr"/>
@@ -17535,7 +17535,7 @@
       </c>
       <c r="P303" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q303" t="inlineStr"/>
@@ -17592,7 +17592,7 @@
       </c>
       <c r="P304" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q304" t="inlineStr"/>
@@ -17649,7 +17649,7 @@
       </c>
       <c r="P305" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q305" t="inlineStr"/>
@@ -17706,7 +17706,7 @@
       </c>
       <c r="P306" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q306" t="inlineStr"/>
@@ -17763,7 +17763,7 @@
       </c>
       <c r="P307" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q307" t="inlineStr"/>
@@ -17820,7 +17820,7 @@
       </c>
       <c r="P308" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q308" t="inlineStr"/>
@@ -17877,7 +17877,7 @@
       </c>
       <c r="P309" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q309" t="inlineStr"/>
@@ -17934,7 +17934,7 @@
       </c>
       <c r="P310" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q310" t="inlineStr"/>
@@ -17991,7 +17991,7 @@
       </c>
       <c r="P311" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q311" t="inlineStr"/>
@@ -18048,7 +18048,7 @@
       </c>
       <c r="P312" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q312" t="inlineStr"/>
@@ -18105,7 +18105,7 @@
       </c>
       <c r="P313" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q313" t="inlineStr"/>
@@ -18162,7 +18162,7 @@
       </c>
       <c r="P314" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q314" t="inlineStr"/>
@@ -18219,7 +18219,7 @@
       </c>
       <c r="P315" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q315" t="inlineStr"/>
@@ -18276,7 +18276,7 @@
       </c>
       <c r="P316" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q316" t="inlineStr"/>
@@ -18333,7 +18333,7 @@
       </c>
       <c r="P317" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q317" t="inlineStr"/>
@@ -18390,7 +18390,7 @@
       </c>
       <c r="P318" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q318" t="inlineStr"/>
@@ -18443,7 +18443,7 @@
       </c>
       <c r="P319" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q319" t="inlineStr"/>
@@ -18500,7 +18500,7 @@
       </c>
       <c r="P320" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q320" t="inlineStr"/>
@@ -18557,7 +18557,7 @@
       </c>
       <c r="P321" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q321" t="inlineStr"/>
@@ -18614,7 +18614,7 @@
       </c>
       <c r="P322" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q322" t="inlineStr"/>
@@ -18671,7 +18671,7 @@
       </c>
       <c r="P323" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q323" t="inlineStr"/>
@@ -18728,7 +18728,7 @@
       </c>
       <c r="P324" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q324" t="inlineStr"/>
@@ -18785,7 +18785,7 @@
       </c>
       <c r="P325" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q325" t="inlineStr"/>
@@ -18842,7 +18842,7 @@
       </c>
       <c r="P326" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q326" t="inlineStr"/>
@@ -18899,7 +18899,7 @@
       </c>
       <c r="P327" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q327" t="inlineStr"/>
@@ -18956,7 +18956,7 @@
       </c>
       <c r="P328" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q328" t="inlineStr"/>
@@ -19013,7 +19013,7 @@
       </c>
       <c r="P329" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q329" t="inlineStr"/>
@@ -19070,7 +19070,7 @@
       </c>
       <c r="P330" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q330" t="inlineStr"/>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="P331" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q331" t="inlineStr"/>
@@ -19176,7 +19176,7 @@
       </c>
       <c r="P332" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q332" t="inlineStr"/>
@@ -19229,7 +19229,7 @@
       </c>
       <c r="P333" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q333" t="inlineStr"/>
@@ -19282,7 +19282,7 @@
       </c>
       <c r="P334" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q334" t="inlineStr"/>
@@ -19335,7 +19335,7 @@
       </c>
       <c r="P335" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q335" t="inlineStr"/>
@@ -19388,7 +19388,7 @@
       </c>
       <c r="P336" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q336" t="inlineStr"/>
@@ -19441,7 +19441,7 @@
       </c>
       <c r="P337" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q337" t="inlineStr"/>
@@ -19494,7 +19494,7 @@
       </c>
       <c r="P338" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q338" t="inlineStr"/>
@@ -19547,7 +19547,7 @@
       </c>
       <c r="P339" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q339" t="inlineStr"/>
@@ -19600,7 +19600,7 @@
       </c>
       <c r="P340" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q340" t="inlineStr"/>
@@ -19653,7 +19653,7 @@
       </c>
       <c r="P341" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q341" t="inlineStr"/>
@@ -19706,7 +19706,7 @@
       </c>
       <c r="P342" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q342" t="inlineStr"/>
@@ -19763,7 +19763,7 @@
       </c>
       <c r="P343" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q343" t="inlineStr"/>
@@ -19816,7 +19816,7 @@
       </c>
       <c r="P344" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q344" t="inlineStr"/>
@@ -19869,7 +19869,7 @@
       </c>
       <c r="P345" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q345" t="inlineStr"/>
@@ -19922,7 +19922,7 @@
       </c>
       <c r="P346" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q346" t="inlineStr"/>
@@ -19975,7 +19975,7 @@
       </c>
       <c r="P347" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q347" t="inlineStr"/>
@@ -20032,7 +20032,7 @@
       </c>
       <c r="P348" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q348" t="inlineStr"/>
@@ -20089,7 +20089,7 @@
       </c>
       <c r="P349" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q349" t="inlineStr"/>
@@ -20142,7 +20142,7 @@
       </c>
       <c r="P350" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q350" t="inlineStr"/>
@@ -20195,7 +20195,7 @@
       </c>
       <c r="P351" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q351" t="inlineStr"/>
@@ -20248,7 +20248,7 @@
       </c>
       <c r="P352" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q352" t="inlineStr"/>
@@ -20305,7 +20305,7 @@
       </c>
       <c r="P353" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q353" t="inlineStr"/>
@@ -20362,7 +20362,7 @@
       </c>
       <c r="P354" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q354" t="inlineStr"/>
@@ -20419,7 +20419,7 @@
       </c>
       <c r="P355" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q355" t="inlineStr"/>
@@ -20476,7 +20476,7 @@
       </c>
       <c r="P356" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q356" t="inlineStr"/>
@@ -20533,7 +20533,7 @@
       </c>
       <c r="P357" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q357" t="inlineStr"/>
@@ -20590,7 +20590,7 @@
       </c>
       <c r="P358" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q358" t="inlineStr"/>
@@ -20647,7 +20647,7 @@
       </c>
       <c r="P359" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q359" t="inlineStr"/>
@@ -20704,7 +20704,7 @@
       </c>
       <c r="P360" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q360" t="inlineStr"/>
@@ -20761,7 +20761,7 @@
       </c>
       <c r="P361" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q361" t="inlineStr"/>
@@ -20818,7 +20818,7 @@
       </c>
       <c r="P362" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q362" t="inlineStr"/>
@@ -20875,7 +20875,7 @@
       </c>
       <c r="P363" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q363" t="inlineStr"/>
@@ -20932,7 +20932,7 @@
       </c>
       <c r="P364" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q364" t="inlineStr"/>
@@ -20989,7 +20989,7 @@
       </c>
       <c r="P365" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q365" t="inlineStr"/>
@@ -21046,7 +21046,7 @@
       </c>
       <c r="P366" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q366" t="inlineStr"/>
@@ -21103,7 +21103,7 @@
       </c>
       <c r="P367" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q367" t="inlineStr"/>
@@ -21160,7 +21160,7 @@
       </c>
       <c r="P368" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q368" t="inlineStr"/>
@@ -21217,7 +21217,7 @@
       </c>
       <c r="P369" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q369" t="inlineStr"/>
@@ -21274,7 +21274,7 @@
       </c>
       <c r="P370" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q370" t="inlineStr"/>
@@ -21331,7 +21331,7 @@
       </c>
       <c r="P371" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q371" t="inlineStr"/>
@@ -21388,7 +21388,7 @@
       </c>
       <c r="P372" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q372" t="inlineStr"/>
@@ -21445,7 +21445,7 @@
       </c>
       <c r="P373" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q373" t="inlineStr"/>
@@ -21502,7 +21502,7 @@
       </c>
       <c r="P374" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q374" t="inlineStr"/>
@@ -21559,7 +21559,7 @@
       </c>
       <c r="P375" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q375" t="inlineStr"/>
@@ -21616,7 +21616,7 @@
       </c>
       <c r="P376" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q376" t="inlineStr"/>
@@ -21673,7 +21673,7 @@
       </c>
       <c r="P377" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q377" t="inlineStr"/>
@@ -21730,7 +21730,7 @@
       </c>
       <c r="P378" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q378" t="inlineStr"/>
@@ -21787,7 +21787,7 @@
       </c>
       <c r="P379" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q379" t="inlineStr"/>
@@ -21844,7 +21844,7 @@
       </c>
       <c r="P380" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q380" t="inlineStr"/>
@@ -21901,7 +21901,7 @@
       </c>
       <c r="P381" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q381" t="inlineStr"/>
@@ -21958,7 +21958,7 @@
       </c>
       <c r="P382" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q382" t="inlineStr"/>
@@ -22015,7 +22015,7 @@
       </c>
       <c r="P383" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q383" t="inlineStr"/>
@@ -22072,7 +22072,7 @@
       </c>
       <c r="P384" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q384" t="inlineStr"/>
@@ -22129,7 +22129,7 @@
       </c>
       <c r="P385" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q385" t="inlineStr"/>
@@ -22186,7 +22186,7 @@
       </c>
       <c r="P386" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q386" t="inlineStr"/>
@@ -22243,7 +22243,7 @@
       </c>
       <c r="P387" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q387" t="inlineStr"/>
@@ -22300,7 +22300,7 @@
       </c>
       <c r="P388" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q388" t="inlineStr"/>
@@ -22357,7 +22357,7 @@
       </c>
       <c r="P389" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q389" t="inlineStr"/>
@@ -22414,7 +22414,7 @@
       </c>
       <c r="P390" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q390" t="inlineStr"/>
@@ -22471,7 +22471,7 @@
       </c>
       <c r="P391" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q391" t="inlineStr"/>
@@ -22528,7 +22528,7 @@
       </c>
       <c r="P392" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q392" t="inlineStr"/>
@@ -22585,7 +22585,7 @@
       </c>
       <c r="P393" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q393" t="inlineStr"/>
@@ -22642,7 +22642,7 @@
       </c>
       <c r="P394" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q394" t="inlineStr"/>
@@ -22699,7 +22699,7 @@
       </c>
       <c r="P395" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q395" t="inlineStr"/>
@@ -22756,7 +22756,7 @@
       </c>
       <c r="P396" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q396" t="inlineStr"/>
@@ -22813,7 +22813,7 @@
       </c>
       <c r="P397" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q397" t="inlineStr"/>
@@ -22870,7 +22870,7 @@
       </c>
       <c r="P398" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q398" t="inlineStr"/>
@@ -22927,7 +22927,7 @@
       </c>
       <c r="P399" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q399" t="inlineStr"/>
@@ -22984,7 +22984,7 @@
       </c>
       <c r="P400" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q400" t="inlineStr"/>
@@ -23041,7 +23041,7 @@
       </c>
       <c r="P401" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q401" t="inlineStr"/>
@@ -23098,7 +23098,7 @@
       </c>
       <c r="P402" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q402" t="inlineStr"/>
@@ -23155,7 +23155,7 @@
       </c>
       <c r="P403" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q403" t="inlineStr"/>
@@ -23212,7 +23212,7 @@
       </c>
       <c r="P404" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q404" t="inlineStr"/>
@@ -23269,7 +23269,7 @@
       </c>
       <c r="P405" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q405" t="inlineStr"/>
@@ -23326,7 +23326,7 @@
       </c>
       <c r="P406" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q406" t="inlineStr"/>
@@ -23383,7 +23383,7 @@
       </c>
       <c r="P407" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q407" t="inlineStr"/>
@@ -23440,7 +23440,7 @@
       </c>
       <c r="P408" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q408" t="inlineStr"/>
@@ -23497,7 +23497,7 @@
       </c>
       <c r="P409" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q409" t="inlineStr"/>
@@ -23554,7 +23554,7 @@
       </c>
       <c r="P410" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q410" t="inlineStr"/>
@@ -23611,7 +23611,7 @@
       </c>
       <c r="P411" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q411" t="inlineStr"/>
@@ -23668,7 +23668,7 @@
       </c>
       <c r="P412" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q412" t="inlineStr"/>
@@ -23725,7 +23725,7 @@
       </c>
       <c r="P413" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q413" t="inlineStr"/>
@@ -23782,7 +23782,7 @@
       </c>
       <c r="P414" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q414" t="inlineStr"/>
@@ -23839,7 +23839,7 @@
       </c>
       <c r="P415" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q415" t="inlineStr"/>
@@ -23896,7 +23896,7 @@
       </c>
       <c r="P416" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q416" t="inlineStr"/>
@@ -23953,7 +23953,7 @@
       </c>
       <c r="P417" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q417" t="inlineStr"/>
@@ -24010,7 +24010,7 @@
       </c>
       <c r="P418" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q418" t="inlineStr"/>
@@ -24067,7 +24067,7 @@
       </c>
       <c r="P419" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q419" t="inlineStr"/>
@@ -24124,7 +24124,7 @@
       </c>
       <c r="P420" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q420" t="inlineStr"/>
@@ -24181,7 +24181,7 @@
       </c>
       <c r="P421" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q421" t="inlineStr"/>
@@ -24238,7 +24238,7 @@
       </c>
       <c r="P422" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q422" t="inlineStr"/>
@@ -24295,7 +24295,7 @@
       </c>
       <c r="P423" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q423" t="inlineStr"/>
@@ -24352,7 +24352,7 @@
       </c>
       <c r="P424" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q424" t="inlineStr"/>
@@ -24409,7 +24409,7 @@
       </c>
       <c r="P425" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q425" t="inlineStr"/>
@@ -24466,7 +24466,7 @@
       </c>
       <c r="P426" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q426" t="inlineStr"/>
@@ -24523,7 +24523,7 @@
       </c>
       <c r="P427" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q427" t="inlineStr"/>
@@ -24576,7 +24576,7 @@
       </c>
       <c r="P428" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q428" t="inlineStr"/>
@@ -24633,7 +24633,7 @@
       </c>
       <c r="P429" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q429" t="inlineStr"/>
@@ -24690,7 +24690,7 @@
       </c>
       <c r="P430" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q430" t="inlineStr"/>
@@ -24743,7 +24743,7 @@
       </c>
       <c r="P431" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q431" t="inlineStr"/>
@@ -24796,7 +24796,7 @@
       </c>
       <c r="P432" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q432" t="inlineStr"/>
@@ -24853,7 +24853,7 @@
       </c>
       <c r="P433" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q433" t="inlineStr"/>
@@ -24910,7 +24910,7 @@
       </c>
       <c r="P434" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q434" t="inlineStr"/>
@@ -24967,7 +24967,7 @@
       </c>
       <c r="P435" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q435" t="inlineStr"/>
@@ -25024,7 +25024,7 @@
       </c>
       <c r="P436" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q436" t="inlineStr"/>
@@ -25081,7 +25081,7 @@
       </c>
       <c r="P437" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q437" t="inlineStr"/>
@@ -25138,7 +25138,7 @@
       </c>
       <c r="P438" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q438" t="inlineStr"/>
@@ -25195,7 +25195,7 @@
       </c>
       <c r="P439" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q439" t="inlineStr"/>
@@ -25252,7 +25252,7 @@
       </c>
       <c r="P440" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q440" t="inlineStr"/>
@@ -25309,7 +25309,7 @@
       </c>
       <c r="P441" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q441" t="inlineStr"/>
@@ -25366,7 +25366,7 @@
       </c>
       <c r="P442" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q442" t="inlineStr"/>
@@ -25419,7 +25419,7 @@
       </c>
       <c r="P443" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q443" t="inlineStr"/>
@@ -25476,7 +25476,7 @@
       </c>
       <c r="P444" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q444" t="inlineStr"/>
@@ -25533,7 +25533,7 @@
       </c>
       <c r="P445" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q445" t="inlineStr"/>
@@ -25590,7 +25590,7 @@
       </c>
       <c r="P446" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q446" t="inlineStr"/>
@@ -25643,7 +25643,7 @@
       </c>
       <c r="P447" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q447" t="inlineStr"/>
@@ -25700,7 +25700,7 @@
       </c>
       <c r="P448" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q448" t="inlineStr"/>
@@ -25757,7 +25757,7 @@
       </c>
       <c r="P449" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q449" t="inlineStr"/>
@@ -25814,7 +25814,7 @@
       </c>
       <c r="P450" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q450" t="inlineStr"/>
@@ -25871,7 +25871,7 @@
       </c>
       <c r="P451" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q451" t="inlineStr"/>
@@ -25928,7 +25928,7 @@
       </c>
       <c r="P452" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q452" t="inlineStr"/>
@@ -25985,7 +25985,7 @@
       </c>
       <c r="P453" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q453" t="inlineStr"/>
@@ -26042,7 +26042,7 @@
       </c>
       <c r="P454" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q454" t="inlineStr"/>
@@ -26099,7 +26099,7 @@
       </c>
       <c r="P455" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q455" t="inlineStr"/>
@@ -26156,7 +26156,7 @@
       </c>
       <c r="P456" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q456" t="inlineStr"/>
@@ -26213,7 +26213,7 @@
       </c>
       <c r="P457" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q457" t="inlineStr"/>
@@ -26270,7 +26270,7 @@
       </c>
       <c r="P458" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q458" t="inlineStr"/>
@@ -26327,7 +26327,7 @@
       </c>
       <c r="P459" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q459" t="inlineStr"/>
@@ -26384,7 +26384,7 @@
       </c>
       <c r="P460" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q460" t="inlineStr"/>
@@ -26441,7 +26441,7 @@
       </c>
       <c r="P461" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q461" t="inlineStr"/>
@@ -26498,7 +26498,7 @@
       </c>
       <c r="P462" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q462" t="inlineStr"/>
@@ -26555,7 +26555,7 @@
       </c>
       <c r="P463" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q463" t="inlineStr"/>
@@ -26612,7 +26612,7 @@
       </c>
       <c r="P464" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q464" t="inlineStr"/>
@@ -26665,7 +26665,7 @@
       </c>
       <c r="P465" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q465" t="inlineStr"/>
@@ -26722,7 +26722,7 @@
       </c>
       <c r="P466" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q466" t="inlineStr"/>
@@ -26779,7 +26779,7 @@
       </c>
       <c r="P467" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q467" t="inlineStr"/>
@@ -26832,7 +26832,7 @@
       </c>
       <c r="P468" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q468" t="inlineStr"/>
@@ -26885,7 +26885,7 @@
       </c>
       <c r="P469" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q469" t="inlineStr"/>
@@ -26938,7 +26938,7 @@
       </c>
       <c r="P470" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q470" t="inlineStr"/>
@@ -26995,7 +26995,7 @@
       </c>
       <c r="P471" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q471" t="inlineStr"/>
@@ -27052,7 +27052,7 @@
       </c>
       <c r="P472" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q472" t="inlineStr"/>
@@ -27109,7 +27109,7 @@
       </c>
       <c r="P473" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q473" t="inlineStr"/>
@@ -27166,7 +27166,7 @@
       </c>
       <c r="P474" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q474" t="inlineStr"/>
@@ -27219,7 +27219,7 @@
       </c>
       <c r="P475" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q475" t="inlineStr"/>
@@ -27272,7 +27272,7 @@
       </c>
       <c r="P476" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q476" t="inlineStr"/>
@@ -27325,7 +27325,7 @@
       </c>
       <c r="P477" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q477" t="inlineStr"/>
@@ -27378,7 +27378,7 @@
       </c>
       <c r="P478" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q478" t="inlineStr"/>
@@ -27431,7 +27431,7 @@
       </c>
       <c r="P479" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q479" t="inlineStr"/>
@@ -27484,7 +27484,7 @@
       </c>
       <c r="P480" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q480" t="inlineStr"/>
@@ -27537,7 +27537,7 @@
       </c>
       <c r="P481" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q481" t="inlineStr"/>
@@ -27590,7 +27590,7 @@
       </c>
       <c r="P482" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q482" t="inlineStr"/>
@@ -27643,7 +27643,7 @@
       </c>
       <c r="P483" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q483" t="inlineStr"/>
@@ -27696,7 +27696,7 @@
       </c>
       <c r="P484" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q484" t="inlineStr"/>
@@ -27749,7 +27749,7 @@
       </c>
       <c r="P485" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q485" t="inlineStr"/>
@@ -27802,7 +27802,7 @@
       </c>
       <c r="P486" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q486" t="inlineStr"/>
@@ -27859,7 +27859,7 @@
       </c>
       <c r="P487" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q487" t="inlineStr"/>
@@ -27916,7 +27916,7 @@
       </c>
       <c r="P488" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q488" t="inlineStr"/>
@@ -27973,7 +27973,7 @@
       </c>
       <c r="P489" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q489" t="inlineStr"/>
@@ -28030,7 +28030,7 @@
       </c>
       <c r="P490" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q490" t="inlineStr"/>
@@ -28087,7 +28087,7 @@
       </c>
       <c r="P491" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q491" t="inlineStr"/>
@@ -28144,7 +28144,7 @@
       </c>
       <c r="P492" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q492" t="inlineStr"/>
@@ -28201,7 +28201,7 @@
       </c>
       <c r="P493" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q493" t="inlineStr"/>
@@ -28258,7 +28258,7 @@
       </c>
       <c r="P494" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q494" t="inlineStr"/>
@@ -28315,7 +28315,7 @@
       </c>
       <c r="P495" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q495" t="inlineStr"/>
@@ -28368,7 +28368,7 @@
       </c>
       <c r="P496" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q496" t="inlineStr"/>
@@ -28421,7 +28421,7 @@
       </c>
       <c r="P497" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q497" t="inlineStr"/>
@@ -28478,7 +28478,7 @@
       </c>
       <c r="P498" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q498" t="inlineStr"/>
@@ -28535,7 +28535,7 @@
       </c>
       <c r="P499" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q499" t="inlineStr"/>
@@ -28588,7 +28588,7 @@
       </c>
       <c r="P500" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q500" t="inlineStr"/>
@@ -28645,7 +28645,7 @@
       </c>
       <c r="P501" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q501" t="inlineStr"/>
@@ -28702,7 +28702,7 @@
       </c>
       <c r="P502" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q502" t="inlineStr"/>
@@ -28759,7 +28759,7 @@
       </c>
       <c r="P503" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q503" t="inlineStr"/>
@@ -28816,7 +28816,7 @@
       </c>
       <c r="P504" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q504" t="inlineStr"/>
@@ -28873,7 +28873,7 @@
       </c>
       <c r="P505" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q505" t="inlineStr"/>
@@ -28930,7 +28930,7 @@
       </c>
       <c r="P506" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q506" t="inlineStr"/>
@@ -28987,7 +28987,7 @@
       </c>
       <c r="P507" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q507" t="inlineStr"/>
@@ -29044,7 +29044,7 @@
       </c>
       <c r="P508" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q508" t="inlineStr"/>
@@ -29101,7 +29101,7 @@
       </c>
       <c r="P509" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q509" t="inlineStr"/>
@@ -29154,7 +29154,7 @@
       </c>
       <c r="P510" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q510" t="inlineStr"/>
@@ -29207,7 +29207,7 @@
       </c>
       <c r="P511" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q511" t="inlineStr"/>
@@ -29260,7 +29260,7 @@
       </c>
       <c r="P512" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q512" t="inlineStr"/>
@@ -29317,7 +29317,7 @@
       </c>
       <c r="P513" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q513" t="inlineStr"/>
@@ -29374,7 +29374,7 @@
       </c>
       <c r="P514" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q514" t="inlineStr"/>
@@ -29431,7 +29431,7 @@
       </c>
       <c r="P515" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q515" t="inlineStr"/>
@@ -29488,7 +29488,7 @@
       </c>
       <c r="P516" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q516" t="inlineStr"/>
@@ -29545,7 +29545,7 @@
       </c>
       <c r="P517" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q517" t="inlineStr"/>
@@ -29598,7 +29598,7 @@
       </c>
       <c r="P518" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="Q518" t="inlineStr"/>
@@ -30235,7 +30235,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2026-07-31T22:25:52.918925</t>
+          <t>2026-08-09T13:55:16.496706</t>
         </is>
       </c>
     </row>

</xml_diff>